<commit_message>
feat: complete email scraping & verification system with modern UI, multi-instance support, and verification pipeline
</commit_message>
<xml_diff>
--- a/WS2.0/downloads/author details/arxiv_hiv_authors.xlsx
+++ b/WS2.0/downloads/author details/arxiv_hiv_authors.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Authors" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Authors'!$A$1:$D$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Authors'!$A$1:$E$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -91,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -99,8 +99,14 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -467,13 +473,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="65" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -494,6 +501,11 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>DOI</t>
         </is>
       </c>
@@ -514,29 +526,39 @@
           <t>nick.williams@nih.gov</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>http://arxiv.org/abs/2304.10023v1</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Evaluating the potential of HIV self-testing to reduce HIV incidence in EHE districts: a modeling study</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Alexander Viguerie</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>alexander.viguerie@uniurb.it</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>http://arxiv.org/abs/2504.15807v1</t>
         </is>
@@ -558,29 +580,39 @@
           <t>adobra@uw.edu</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>http://arxiv.org/abs/2512.11159v1</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Quantum Approximate Optimization Algorithm for Spatiotemporal Forecasting of HIV Clusters</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Roosand</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>roosand@merrimack.edu</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>http://arxiv.org/abs/2507.00848v1</t>
         </is>
@@ -602,29 +634,39 @@
           <t>saif.nirzhor@utsouthwestern.edu</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>http://arxiv.org/abs/2507.00848v1</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Quantum Approximate Optimization Algorithm for Spatiotemporal Forecasting of HIV Clusters</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Rubayat Khan</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>rubayat.khan@unmc.edu</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>http://arxiv.org/abs/2507.00848v1</t>
         </is>
@@ -646,29 +688,39 @@
           <t>fahmida@tekurai.com</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>http://arxiv.org/abs/2507.00848v1</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Quantum Approximate Optimization Algorithm for Spatiotemporal Forecasting of HIV Clusters</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Haider</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>haider@uga.edu</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>http://arxiv.org/abs/2507.00848v1</t>
         </is>
@@ -690,29 +742,39 @@
           <t>wenlong@psu.edu</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>http://arxiv.org/abs/2309.02430v2</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>A Likelihood Approach to Incorporating Self-Report Data in HIV Recency Classification</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Danping Liu</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>danping.liu@nih.gov</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>http://arxiv.org/abs/2309.02430v2</t>
         </is>
@@ -734,29 +796,39 @@
           <t>lub14@psu.edu</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>http://arxiv.org/abs/2309.02430v2</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>A Likelihood Approach to Incorporating Self-Report Data in HIV Recency Classification</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>rzli@psu.edu</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>http://arxiv.org/abs/2309.02430v2</t>
         </is>
@@ -778,29 +850,39 @@
           <t>jhuwa@lighthouse.org.mw</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1145/3613904.3642245</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>HIV Client Perspectives on Digital Health in Malawi</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>ckamamia@lighthouse.org.mw</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>https://doi.org/10.1145/3613904.3642245</t>
         </is>
@@ -822,14 +904,19 @@
           <t>xjm9@cdc.gov</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>http://arxiv.org/abs/2404.04222v1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D16"/>
+  <autoFilter ref="A1:E16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>